<commit_message>
fix: correct Zimbabwe Portuguese spelling
</commit_message>
<xml_diff>
--- a/info/paises/africa/zimbabue/coins-availability.xlsx
+++ b/info/paises/africa/zimbabue/coins-availability.xlsx
@@ -78,7 +78,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›2024 - 2024</t>
+          <t>Zimbabué›República do Zimbabué›2024 - 2024</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -100,7 +100,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›2024 - 2024</t>
+          <t>Zimbabué›República do Zimbabué›2024 - 2024</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -122,7 +122,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›2024 - 2024</t>
+          <t>Zimbabué›República do Zimbabué›2024 - 2024</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -144,7 +144,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›2014 - 2023</t>
+          <t>Zimbabué›República do Zimbabué›2014 - 2023</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -166,7 +166,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›2014 - 2023</t>
+          <t>Zimbabué›República do Zimbabué›2014 - 2023</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -188,7 +188,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›2014 - 2023</t>
+          <t>Zimbabué›República do Zimbabué›2014 - 2023</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -210,7 +210,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›2014 - 2023</t>
+          <t>Zimbabué›República do Zimbabué›2014 - 2023</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -232,7 +232,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›2014 - 2023</t>
+          <t>Zimbabué›República do Zimbabué›2014 - 2023</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -254,7 +254,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›2014 - 2023</t>
+          <t>Zimbabué›República do Zimbabué›2014 - 2023</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -276,7 +276,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›2014 - 2023</t>
+          <t>Zimbabué›República do Zimbabué›2014 - 2023</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -298,7 +298,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›1980 - 2009</t>
+          <t>Zimbabué›República do Zimbabué›1980 - 2009</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -320,7 +320,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›1980 - 2009</t>
+          <t>Zimbabué›República do Zimbabué›1980 - 2009</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -342,7 +342,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›1980 - 2009</t>
+          <t>Zimbabué›República do Zimbabué›1980 - 2009</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -364,7 +364,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›1980 - 2009</t>
+          <t>Zimbabué›República do Zimbabué›1980 - 2009</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -386,7 +386,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›1980 - 2009</t>
+          <t>Zimbabué›República do Zimbabué›1980 - 2009</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -408,7 +408,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›1980 - 2009</t>
+          <t>Zimbabué›República do Zimbabué›1980 - 2009</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -430,7 +430,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›1980 - 2009</t>
+          <t>Zimbabué›República do Zimbabué›1980 - 2009</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -452,7 +452,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›1980 - 2009</t>
+          <t>Zimbabué›República do Zimbabué›1980 - 2009</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -474,7 +474,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›1980 - 2009</t>
+          <t>Zimbabué›República do Zimbabué›1980 - 2009</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -496,7 +496,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›1980 - 2009</t>
+          <t>Zimbabué›República do Zimbabué›1980 - 2009</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -518,7 +518,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›1980 - 2009</t>
+          <t>Zimbabué›República do Zimbabué›1980 - 2009</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -540,7 +540,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›1980 - 2009</t>
+          <t>Zimbabué›República do Zimbabué›1980 - 2009</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -562,7 +562,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›1980 - 2009</t>
+          <t>Zimbabué›República do Zimbabué›1980 - 2009</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -584,7 +584,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›1980 - 2009</t>
+          <t>Zimbabué›República do Zimbabué›1980 - 2009</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -606,7 +606,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›1980 - 2009</t>
+          <t>Zimbabué›República do Zimbabué›1980 - 2009</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -628,7 +628,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Zimbábue›República do Zimbábue›1980 - 2009</t>
+          <t>Zimbabué›República do Zimbabué›1980 - 2009</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">

</xml_diff>